<commit_message>
A7.1: tệp nhập Sheet đánh dấu đã kiểm tra các dòng còn lại của cụm
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013nDsfVobQsuvYZZzABT4iC
</commit_message>
<xml_diff>
--- a/tools/ra/xinyu-noi-dung.xlsx
+++ b/tools/ra/xinyu-noi-dung.xlsx
@@ -1828,7 +1828,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C10">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C11">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C12">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C13">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C14">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C15">
@@ -3130,7 +3130,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C16">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C17">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C18">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C19">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C30">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C31">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C42">
@@ -7148,7 +7148,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C63">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C67">
@@ -7482,7 +7482,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C71">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C73">
@@ -7817,7 +7817,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C80">
@@ -7926,7 +7926,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C83">
@@ -8137,7 +8137,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C89">
@@ -9038,7 +9038,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C115">
@@ -9393,7 +9393,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C125">
@@ -9659,7 +9659,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C132">
@@ -9702,7 +9702,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C133">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C135">
@@ -9920,7 +9920,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C139">
@@ -9958,7 +9958,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C140">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C145">
@@ -10186,7 +10186,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C146">
@@ -10229,7 +10229,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C147">
@@ -10343,7 +10343,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C150">
@@ -10386,7 +10386,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C151">
@@ -10467,7 +10467,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C153">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C155">
@@ -10581,7 +10581,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C156">
@@ -10994,7 +10994,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C167">
@@ -11136,7 +11136,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C171">
@@ -11179,7 +11179,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C172">
@@ -11534,7 +11534,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C182">
@@ -11610,7 +11610,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C184">
@@ -11719,7 +11719,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C187">
@@ -12084,7 +12084,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C197">
@@ -12226,7 +12226,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C201">
@@ -12302,7 +12302,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C203">
@@ -12378,7 +12378,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C205">
@@ -12454,7 +12454,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C207">
@@ -12997,7 +12997,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C222">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C223">
@@ -13309,7 +13309,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C231">
@@ -13598,7 +13598,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C239">
@@ -13925,7 +13925,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C248">
@@ -14001,7 +14001,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C250">
@@ -14178,7 +14178,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C254">
@@ -14368,7 +14368,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C259">
@@ -14817,7 +14817,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C272">
@@ -15101,7 +15101,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C280">
@@ -15177,7 +15177,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C282">
@@ -15423,7 +15423,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C289">
@@ -15742,7 +15742,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C297">
@@ -15818,7 +15818,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C299">
@@ -16229,7 +16229,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C16">
@@ -16436,7 +16436,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C28">
@@ -16507,7 +16507,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C31">
@@ -16560,7 +16560,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C33">
@@ -16679,7 +16679,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C39">
@@ -16897,7 +16897,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C51">
@@ -16968,7 +16968,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C54">
@@ -17024,7 +17024,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C56">
@@ -17060,7 +17060,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C57">
@@ -17143,7 +17143,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C61">
@@ -17232,7 +17232,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C65">
@@ -17273,7 +17273,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C66">
@@ -17362,7 +17362,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C70">
@@ -17481,7 +17481,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C76">
@@ -17651,7 +17651,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C85">
@@ -17791,7 +17791,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C92">
@@ -17913,7 +17913,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C98">
@@ -18078,7 +18078,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C107">
@@ -18179,7 +18179,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C112">
@@ -18253,7 +18253,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C115">
@@ -18324,7 +18324,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C118">
@@ -18380,7 +18380,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C120">
@@ -18418,7 +18418,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C121">
@@ -18469,7 +18469,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C123">
@@ -18525,7 +18525,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C125">
@@ -18563,7 +18563,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C126">
@@ -18596,7 +18596,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C127">
@@ -18655,7 +18655,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C129">
@@ -18708,7 +18708,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C131">
@@ -18749,7 +18749,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C132">
@@ -18925,7 +18925,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C142">
@@ -18996,7 +18996,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C145">
@@ -19037,7 +19037,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C146">
@@ -19162,7 +19162,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C152">
@@ -19200,7 +19200,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C153">
@@ -19241,7 +19241,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C154">
@@ -19282,7 +19282,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C155">
@@ -19351,7 +19351,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C158">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C159">
@@ -19472,7 +19472,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C163">
@@ -19576,7 +19576,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C168">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C169">
@@ -19686,7 +19686,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C172">
@@ -19742,7 +19742,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C174">
@@ -19861,7 +19861,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C180">
@@ -19957,7 +19957,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C185">
@@ -19993,7 +19993,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C186">
@@ -20031,7 +20031,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C187">
@@ -20138,7 +20138,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C192">
@@ -20222,7 +20222,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C196">
@@ -20336,7 +20336,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C202">
@@ -20422,7 +20422,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C206">
@@ -20470,7 +20470,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C208">
@@ -20559,7 +20559,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C212">
@@ -20628,7 +20628,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C215">
@@ -20681,7 +20681,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C217">
@@ -20747,7 +20747,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C220">
@@ -20813,7 +20813,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C223">
@@ -20917,7 +20917,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C228">
@@ -20998,7 +20998,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C232">
@@ -21069,7 +21069,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C235">
@@ -21122,7 +21122,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C237">
@@ -21226,7 +21226,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C242">
@@ -21297,7 +21297,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C245">
@@ -21353,7 +21353,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C247">
@@ -21487,7 +21487,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C3">
@@ -21552,7 +21552,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C5">
@@ -21617,7 +21617,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C7">
@@ -21682,7 +21682,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C9">
@@ -21727,7 +21727,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C10">
@@ -21772,7 +21772,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C11">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C16">
@@ -21942,7 +21942,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C17">
@@ -22027,7 +22027,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C20">
@@ -22072,7 +22072,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C21">
@@ -22117,7 +22117,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C22">
@@ -22202,7 +22202,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C25">
@@ -22327,7 +22327,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C30">
@@ -22372,7 +22372,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C31">
@@ -22417,7 +22417,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C32">
@@ -22482,7 +22482,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C34">
@@ -22547,7 +22547,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C36">
@@ -22632,7 +22632,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C39">
@@ -22677,7 +22677,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C40">
@@ -22762,7 +22762,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C43">
@@ -22807,7 +22807,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C44">
@@ -22917,7 +22917,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C47">
@@ -22962,7 +22962,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C48">
@@ -23007,7 +23007,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C49">
@@ -23052,7 +23052,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C50">
@@ -23137,7 +23137,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C53">
@@ -23908,7 +23908,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -23945,7 +23945,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -23982,7 +23982,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -24019,7 +24019,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -24056,7 +24056,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -24093,7 +24093,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -24130,7 +24130,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -24167,7 +24167,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -24204,7 +24204,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -24241,7 +24241,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -24278,7 +24278,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -24315,7 +24315,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -24352,7 +24352,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -24389,7 +24389,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -24426,7 +24426,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -24463,7 +24463,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -24500,7 +24500,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -24537,7 +24537,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -24574,7 +24574,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -24611,7 +24611,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -24648,7 +24648,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -24685,7 +24685,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -24722,7 +24722,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -24759,7 +24759,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -24796,7 +24796,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -24833,7 +24833,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -24870,7 +24870,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -24907,7 +24907,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -24944,7 +24944,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -24981,7 +24981,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -25018,7 +25018,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -25055,7 +25055,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -25092,7 +25092,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -25129,7 +25129,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -25166,7 +25166,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -25240,7 +25240,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -25277,7 +25277,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -25314,7 +25314,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -25351,7 +25351,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -25388,7 +25388,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -25425,7 +25425,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -25462,7 +25462,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -25499,7 +25499,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -25536,7 +25536,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -25573,7 +25573,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -25610,7 +25610,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -25647,7 +25647,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -25684,7 +25684,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -25721,7 +25721,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -25758,7 +25758,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -25795,7 +25795,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -25832,7 +25832,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -25869,7 +25869,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -25906,7 +25906,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -25943,7 +25943,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -25980,7 +25980,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -26017,7 +26017,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -26054,7 +26054,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -26091,7 +26091,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -26128,7 +26128,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -26165,7 +26165,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -26202,7 +26202,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -26239,7 +26239,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -26276,7 +26276,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -26313,7 +26313,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -26350,7 +26350,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -26387,7 +26387,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -26424,7 +26424,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -26461,7 +26461,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -26498,7 +26498,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -26535,7 +26535,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -26572,7 +26572,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -26609,7 +26609,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -26646,7 +26646,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -26683,7 +26683,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -26720,7 +26720,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -26757,7 +26757,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -26794,7 +26794,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -26831,7 +26831,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -26868,7 +26868,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -26905,7 +26905,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -26942,7 +26942,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -26979,7 +26979,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -27016,7 +27016,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -31870,7 +31870,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -31942,7 +31942,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -32009,7 +32009,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -32081,7 +32081,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -32148,7 +32148,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -32215,7 +32215,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -32287,7 +32287,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -32359,7 +32359,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -32426,7 +32426,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -32493,7 +32493,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -32565,7 +32565,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -32632,7 +32632,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -32704,7 +32704,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -32776,7 +32776,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -32843,7 +32843,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -32910,7 +32910,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -32977,7 +32977,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -33044,7 +33044,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -33111,7 +33111,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -33255,7 +33255,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -33322,7 +33322,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -33389,7 +33389,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -33461,7 +33461,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -33528,7 +33528,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -33595,7 +33595,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -33667,7 +33667,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -33734,7 +33734,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -33801,7 +33801,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -33873,7 +33873,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -33940,7 +33940,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -34012,7 +34012,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -34084,7 +34084,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -34151,7 +34151,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -34218,7 +34218,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -34285,7 +34285,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -34357,7 +34357,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -34429,7 +34429,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -34501,7 +34501,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -34568,7 +34568,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -34635,7 +34635,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -34707,7 +34707,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -34774,7 +34774,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -34846,7 +34846,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -34918,7 +34918,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -34985,7 +34985,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -35052,7 +35052,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -35124,7 +35124,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -35191,7 +35191,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -35263,7 +35263,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -35330,7 +35330,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -35402,7 +35402,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -35469,7 +35469,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -35536,7 +35536,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -35608,7 +35608,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -35675,7 +35675,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -35747,7 +35747,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -35819,7 +35819,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -35886,7 +35886,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -35953,7 +35953,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -36020,7 +36020,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -36092,7 +36092,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -36159,7 +36159,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t xml:space="preserve">nháp</t>
+          <t xml:space="preserve">đã kiểm tra</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">

</xml_diff>